<commit_message>
infra: adiciona ESSENCIAL standalone ao modelo e cria operacao PB_DISTRIB
- OPERACOES/_MODELO_OPERACAO/ESSENCIAL/ criada com Python 3.12
  embeddable proprio (porta 8601, entidade_auditada: null, historico
  zerado) — modelo agora totalmente independente de geraldo_2020_2024.
- OPERACOES/PB_DISTRIB/ criada pelo usuario como primeira operacao real
  alem de Geraldo (a partir do modelo).
- memoria/2026-07-01.md: registro do dia com decisoes e validacao.
</commit_message>
<xml_diff>
--- a/fluxo.xlsx
+++ b/fluxo.xlsx
@@ -16,10 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>BAT</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>PASTA OPERAÇÕES</t>
   </si>
@@ -36,10 +33,28 @@
     <t>PASTA PRINCIPAL</t>
   </si>
   <si>
-    <t>SUBPASTAS  E APLICAÇÕES</t>
-  </si>
-  <si>
-    <t>USUÁRIO ESCOLHE A OPERAÇÃO E BAT EXECUTA A CARGA</t>
+    <t>bat</t>
+  </si>
+  <si>
+    <t>fase 1</t>
+  </si>
+  <si>
+    <t>aciona o bat</t>
+  </si>
+  <si>
+    <t>fase2</t>
+  </si>
+  <si>
+    <t>fase</t>
+  </si>
+  <si>
+    <t>bat gera painel operaração ativa  e quantidades de arquivos por pasta e botão carregar dados</t>
+  </si>
+  <si>
+    <t>depois de carregados os dados, aí sim gera dados de presa auditada, quatidade de registros ET, EP e DECLARAÇÕES</t>
+  </si>
+  <si>
+    <t>perações com pastas para receber dados. Cada operação conterá um bat</t>
   </si>
 </sst>
 </file>
@@ -75,8 +90,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -378,52 +396,71 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="45.7109375" customWidth="1"/>
-    <col min="3" max="3" width="52.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" style="1" customWidth="1"/>
+    <col min="3" max="4" width="21.85546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="18.42578125" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="120" x14ac:dyDescent="0.25">
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>4</v>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>